<commit_message>
tecan channel names no longer have "OD "
</commit_message>
<xml_diff>
--- a/test/inputs/tecan.xlsx
+++ b/test/inputs/tecan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3627A845-3FEA-BB4D-80A9-61B098FF8183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B5D929-BAF2-AE42-A1F7-4EDEA61E5984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19420" yWindow="7480" windowWidth="18980" windowHeight="9440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
@@ -87,7 +87,7 @@
     <t>tecan</t>
   </si>
   <si>
-    <t>OD 600,OD 700,GFP</t>
+    <t>600,700,GFP</t>
   </si>
 </sst>
 </file>

</xml_diff>